<commit_message>
new API from Ritik
</commit_message>
<xml_diff>
--- a/uploads/attendance/696c72aa0b1580f87ebbe9b3/2026/02.xlsx
+++ b/uploads/attendance/696c72aa0b1580f87ebbe9b3/2026/02.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="26">
   <si>
     <t>Enrollment No</t>
   </si>
@@ -19,19 +19,58 @@
     <t>Student Name</t>
   </si>
   <si>
-    <t>2026-02-01</t>
-  </si>
-  <si>
-    <t>2026-02-06</t>
+    <t>2026-02-15</t>
   </si>
   <si>
     <t>MCA102</t>
   </si>
   <si>
-    <t>18:52-16:32</t>
-  </si>
-  <si>
-    <t>20:39-16:32</t>
+    <t>18:28-19:36</t>
+  </si>
+  <si>
+    <t>19:24-19:36</t>
+  </si>
+  <si>
+    <t>19:24-19:42</t>
+  </si>
+  <si>
+    <t>18:28-19:42</t>
+  </si>
+  <si>
+    <t>18:28-19:43</t>
+  </si>
+  <si>
+    <t>18:28-19:45</t>
+  </si>
+  <si>
+    <t>18:28-19:47</t>
+  </si>
+  <si>
+    <t>19:24-19:47</t>
+  </si>
+  <si>
+    <t>19:24-19:48</t>
+  </si>
+  <si>
+    <t>18:28-19:50</t>
+  </si>
+  <si>
+    <t>19:24-19:51</t>
+  </si>
+  <si>
+    <t>18:28-19:55</t>
+  </si>
+  <si>
+    <t>19:24-19:55</t>
+  </si>
+  <si>
+    <t>19:24-19:03</t>
+  </si>
+  <si>
+    <t>19:24-19:04</t>
+  </si>
+  <si>
+    <t>19:24-19:07</t>
   </si>
   <si>
     <t>MCA123</t>
@@ -426,10 +465,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -440,35 +479,161 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" t="s">
+        <v>2</v>
+      </c>
+      <c r="L1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N1" t="s">
+        <v>2</v>
+      </c>
+      <c r="O1" t="s">
+        <v>2</v>
+      </c>
+      <c r="P1" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>2</v>
+      </c>
+      <c r="R1" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" t="s">
+        <v>3</v>
+      </c>
+      <c r="O2" t="s">
+        <v>3</v>
+      </c>
+      <c r="P2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>3</v>
+      </c>
+      <c r="R2" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3"/>
       <c r="B3"/>
       <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>6</v>
       </c>
+      <c r="F3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" t="s">
+        <v>14</v>
+      </c>
+      <c r="N3" t="s">
+        <v>15</v>
+      </c>
+      <c r="O3" t="s">
+        <v>16</v>
+      </c>
+      <c r="P3" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>18</v>
+      </c>
+      <c r="R3" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -476,13 +641,55 @@
       <c r="D4">
         <v>0</v>
       </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -490,13 +697,55 @@
       <c r="D5">
         <v>0</v>
       </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -504,13 +753,55 @@
       <c r="D6">
         <v>0</v>
       </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -518,19 +809,103 @@
       <c r="D7">
         <v>0</v>
       </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
         <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>1</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8">
+        <v>1</v>
+      </c>
+      <c r="R8">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>